<commit_message>
Add Phone field/column to Users page
UsersPage.tsx: Phone input on the create/edit form, a Phone column on the
list table, included in search, and the bulk-import help text updated to
mention the new template column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/User_Master_Import_Template.xlsx
+++ b/frontend/public/templates/User_Master_Import_Template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,6 +417,9 @@
         <v>Function Tag</v>
       </c>
       <c r="F1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="G1" t="str">
         <v>Warehouse Code(s)</v>
       </c>
     </row>
@@ -437,6 +440,9 @@
         <v>Inbound Sup</v>
       </c>
       <c r="F2" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G2" t="str">
         <v>TN01</v>
       </c>
     </row>
@@ -457,19 +463,22 @@
         <v>Picking</v>
       </c>
       <c r="F3" t="str">
+        <v>9123456789</v>
+      </c>
+      <c r="G3" t="str">
         <v>TN01;MH02</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -539,18 +548,29 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="B7" t="str">
+        <v>No</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Contact number, used for SMS/WhatsApp notifications once that capability is wired up. Not validated for format today.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Warehouse Code(s)</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B8" t="str">
         <v>Required for every role except Company Admin</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C8" t="str">
         <v>One or more existing Warehouse Location Codes for this company, separated by a comma or semicolon (e.g. "TN01;MH02"). You can only assign warehouses you yourself have access to.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>